<commit_message>
docs: update progress report and workplan
</commit_message>
<xml_diff>
--- a/documentation/srs/UIRI_IMS_Updated_Workplan.xlsx
+++ b/documentation/srs/UIRI_IMS_Updated_Workplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\uiri-ims\documentation\srs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259534EA-6937-4B31-9B8D-E5468C435218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A2C8FE-8527-4312-A909-D8A33F447755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4665" yWindow="2985" windowWidth="15375" windowHeight="8325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectSchedule" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="85">
   <si>
     <t>TASK</t>
   </si>
@@ -178,9 +178,6 @@
     <t>Keith &amp; Deo</t>
   </si>
   <si>
-    <t>Security requirements and audit review</t>
-  </si>
-  <si>
     <t>Phase 3: Database Design and Documentation</t>
   </si>
   <si>
@@ -196,9 +193,6 @@
     <t>Logical ERD and 3NF normalization</t>
   </si>
   <si>
-    <t>Extended ERD review and corrections</t>
-  </si>
-  <si>
     <t>Phase 4: Database Implementation</t>
   </si>
   <si>
@@ -208,57 +202,6 @@
     <t>Primary keys, foreign keys and constraints</t>
   </si>
   <si>
-    <t>Campus, department and category seed data</t>
-  </si>
-  <si>
-    <t>Authentication and RBAC tables</t>
-  </si>
-  <si>
-    <t>Database integrity review</t>
-  </si>
-  <si>
-    <t>Phase 5: Application Modules, Testing and Documentation</t>
-  </si>
-  <si>
-    <t>Inventory item and asset instance module</t>
-  </si>
-  <si>
-    <t>Stock in, stock out and transfer module</t>
-  </si>
-  <si>
-    <t>Supplier, dashboard and reports module</t>
-  </si>
-  <si>
-    <t>Security, audit trail and validation checks</t>
-  </si>
-  <si>
-    <t>System testing and correction</t>
-  </si>
-  <si>
-    <t>Phase 6: Presentation and Final Submission</t>
-  </si>
-  <si>
-    <t>Final proposal and SRS packaging</t>
-  </si>
-  <si>
-    <t>ERD and UML diagrams finalization in Visio</t>
-  </si>
-  <si>
-    <t>Deo</t>
-  </si>
-  <si>
-    <t>User manual and final project report</t>
-  </si>
-  <si>
-    <t>Presentation slides and demonstration script</t>
-  </si>
-  <si>
-    <t>Supervisor presentation and handover</t>
-  </si>
-  <si>
-    <t>UIRI Inventory Management System Work Plan</t>
-  </si>
-  <si>
     <t>Project</t>
   </si>
   <si>
@@ -289,21 +232,12 @@
     <t>Keith Paul Kato</t>
   </si>
   <si>
-    <t>Lead reporter, database design, normalization, schema implementation</t>
-  </si>
-  <si>
     <t>Komukama Tracy</t>
   </si>
   <si>
-    <t>Requirements, SRS, documentation, supplier and report module support</t>
-  </si>
-  <si>
     <t>Atuhiire Deo Kamate</t>
   </si>
   <si>
-    <t>Data dictionary, UML diagrams, testing and dashboard support</t>
-  </si>
-  <si>
     <t>Supervisor</t>
   </si>
   <si>
@@ -320,6 +254,75 @@
   </si>
   <si>
     <t>Database Project Team:</t>
+  </si>
+  <si>
+    <t>Phase 5: Application Modules, Security Hardening and Deployment</t>
+  </si>
+  <si>
+    <t>Phase 6: Testing, Documentation and Final Submission</t>
+  </si>
+  <si>
+    <t>Security requirements, session policy and audit review</t>
+  </si>
+  <si>
+    <t>Extended ERD review and implementation corrections</t>
+  </si>
+  <si>
+    <t>Campus, department, category and inventory seed data</t>
+  </si>
+  <si>
+    <t>Tracy &amp; Keith</t>
+  </si>
+  <si>
+    <t>Authentication, RBAC and session security tables</t>
+  </si>
+  <si>
+    <t>Database integrity, audit and deployment readiness review</t>
+  </si>
+  <si>
+    <t>Inventory item registration, details preview and item-print workflow</t>
+  </si>
+  <si>
+    <t>Stock-in, stock-out, adjustment and recent movement panels</t>
+  </si>
+  <si>
+    <t>Supplier, management tables, delete confirmations and UI consistency</t>
+  </si>
+  <si>
+    <t>Dashboard, analytics, reports and table visual standardisation</t>
+  </si>
+  <si>
+    <t>Idle timeout, landing-page logout behaviour and Alwaysdata deployment</t>
+  </si>
+  <si>
+    <t>Evidence screenshots, progress report update and workplan appendix image</t>
+  </si>
+  <si>
+    <t>Final UAT checklist for authentication, inventory, stock, reports and audit trail</t>
+  </si>
+  <si>
+    <t>Deo &amp; Keith</t>
+  </si>
+  <si>
+    <t>User manual and final project report packaging</t>
+  </si>
+  <si>
+    <t>Presentation slides, demonstration script and supervisor review</t>
+  </si>
+  <si>
+    <t>Supervisor presentation, handover and final corrections</t>
+  </si>
+  <si>
+    <t>UIRI Inventory Management System Work Plan - Updated 19 July 2026</t>
+  </si>
+  <si>
+    <t>Lead reporter; database design; PHP/MySQL implementation; security hardening; Alwaysdata deployment coordination.</t>
+  </si>
+  <si>
+    <t>Requirements and SRS review; documentation quality control; user workflow validation and report evidence support.</t>
+  </si>
+  <si>
+    <t>Data dictionary, UML/database validation, test support and final UAT evidence preparation.</t>
   </si>
 </sst>
 </file>
@@ -1432,6 +1435,114 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1BF44AF-1AC0-E7EA-4A5A-3409B64C9809}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EBEA110-3E52-7FC6-102F-6D60E09B97D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9810750"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1642,13 +1753,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="32" style="13" customWidth="1"/>
-    <col min="3" max="3" width="18" style="13" customWidth="1"/>
-    <col min="4" max="4" width="10" style="13" customWidth="1"/>
-    <col min="5" max="5" width="10" style="21" customWidth="1"/>
-    <col min="6" max="6" width="10" style="13" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" style="13" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="13" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="21" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="13" customWidth="1"/>
     <col min="7" max="7" width="2.7109375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="6" style="13" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" style="13" customWidth="1"/>
     <col min="9" max="50" width="3" customWidth="1"/>
     <col min="51" max="64" width="2.5703125" style="13" customWidth="1"/>
     <col min="65" max="65" width="9.140625" style="13" customWidth="1"/>
@@ -1701,14 +1812,14 @@
     </row>
     <row r="3" spans="1:64" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="C3"/>
       <c r="D3" s="19" t="s">
         <v>15</v>
       </c>
       <c r="E3" s="129">
-        <v>46201</v>
+        <v>46222</v>
       </c>
       <c r="F3" s="130"/>
     </row>
@@ -1721,7 +1832,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F4"/>
       <c r="I4" s="123">
@@ -3086,7 +3197,7 @@
       <c r="BK17" s="42"/>
       <c r="BL17" s="42"/>
     </row>
-    <row r="18" spans="1:64" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
       <c r="A18" s="19"/>
       <c r="B18" s="67" t="s">
         <v>34</v>
@@ -3165,27 +3276,27 @@
       <c r="BK18" s="42"/>
       <c r="BL18" s="42"/>
     </row>
-    <row r="19" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="19"/>
       <c r="B19" s="67" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="C19" s="68" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="D19" s="110">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="E19" s="63">
         <v>46200</v>
       </c>
       <c r="F19" s="113">
-        <v>46201</v>
+        <v>46222</v>
       </c>
       <c r="G19" s="28"/>
       <c r="H19" s="64">
-        <f t="shared" si="6"/>
-        <v>2</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>23</v>
       </c>
       <c r="I19" s="42"/>
       <c r="J19" s="42"/>
@@ -3244,10 +3355,10 @@
       <c r="BK19" s="42"/>
       <c r="BL19" s="42"/>
     </row>
-    <row r="20" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="19"/>
       <c r="B20" s="70" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="71"/>
       <c r="D20" s="106"/>
@@ -3315,10 +3426,10 @@
       <c r="BK20" s="42"/>
       <c r="BL20" s="42"/>
     </row>
-    <row r="21" spans="1:64" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="19"/>
       <c r="B21" s="76" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C21" s="77" t="s">
         <v>26</v>
@@ -3394,10 +3505,10 @@
       <c r="BK21" s="42"/>
       <c r="BL21" s="42"/>
     </row>
-    <row r="22" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="19"/>
       <c r="B22" s="76" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="77" t="s">
         <v>24</v>
@@ -3473,10 +3584,10 @@
       <c r="BK22" s="42"/>
       <c r="BL22" s="42"/>
     </row>
-    <row r="23" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="19"/>
       <c r="B23" s="76" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="77" t="s">
         <v>35</v>
@@ -3552,10 +3663,10 @@
       <c r="BK23" s="42"/>
       <c r="BL23" s="42"/>
     </row>
-    <row r="24" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="19"/>
       <c r="B24" s="76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C24" s="77" t="s">
         <v>26</v>
@@ -3631,16 +3742,16 @@
       <c r="BK24" s="42"/>
       <c r="BL24" s="42"/>
     </row>
-    <row r="25" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="19"/>
       <c r="B25" s="76" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="C25" s="77" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="110">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E25" s="72">
         <v>46207</v>
@@ -3650,7 +3761,7 @@
       </c>
       <c r="G25" s="28"/>
       <c r="H25" s="73">
-        <f t="shared" si="6"/>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>2</v>
       </c>
       <c r="I25" s="42"/>
@@ -3710,10 +3821,10 @@
       <c r="BK25" s="42"/>
       <c r="BL25" s="42"/>
     </row>
-    <row r="26" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="19"/>
       <c r="B26" s="79" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C26" s="80"/>
       <c r="D26" s="107"/>
@@ -3781,10 +3892,10 @@
       <c r="BK26" s="42"/>
       <c r="BL26" s="42"/>
     </row>
-    <row r="27" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="19"/>
       <c r="B27" s="85" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C27" s="86" t="s">
         <v>26</v>
@@ -3860,10 +3971,10 @@
       <c r="BK27" s="42"/>
       <c r="BL27" s="42"/>
     </row>
-    <row r="28" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="19"/>
       <c r="B28" s="85" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C28" s="86" t="s">
         <v>35</v>
@@ -3939,27 +4050,27 @@
       <c r="BK28" s="42"/>
       <c r="BL28" s="42"/>
     </row>
-    <row r="29" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="19"/>
       <c r="B29" s="85" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C29" s="86" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="D29" s="110">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="E29" s="81">
         <v>46211</v>
       </c>
       <c r="F29" s="117">
-        <v>46212</v>
+        <v>46222</v>
       </c>
       <c r="G29" s="28"/>
       <c r="H29" s="82">
-        <f t="shared" si="6"/>
-        <v>2</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>12</v>
       </c>
       <c r="I29" s="42"/>
       <c r="J29" s="42"/>
@@ -4018,27 +4129,27 @@
       <c r="BK29" s="42"/>
       <c r="BL29" s="42"/>
     </row>
-    <row r="30" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="19"/>
       <c r="B30" s="85" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="C30" s="86" t="s">
         <v>26</v>
       </c>
       <c r="D30" s="110">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="E30" s="81">
         <v>46212</v>
       </c>
       <c r="F30" s="117">
-        <v>46213</v>
+        <v>46222</v>
       </c>
       <c r="G30" s="28"/>
       <c r="H30" s="82">
-        <f t="shared" si="6"/>
-        <v>2</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>11</v>
       </c>
       <c r="I30" s="42"/>
       <c r="J30" s="42"/>
@@ -4097,27 +4208,27 @@
       <c r="BK30" s="42"/>
       <c r="BL30" s="42"/>
     </row>
-    <row r="31" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="19"/>
       <c r="B31" s="85" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="C31" s="86" t="s">
         <v>20</v>
       </c>
       <c r="D31" s="110">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E31" s="81">
         <v>46213</v>
       </c>
       <c r="F31" s="117">
-        <v>46215</v>
+        <v>46222</v>
       </c>
       <c r="G31" s="28"/>
       <c r="H31" s="82">
-        <f t="shared" si="6"/>
-        <v>3</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>10</v>
       </c>
       <c r="I31" s="42"/>
       <c r="J31" s="42"/>
@@ -4176,10 +4287,10 @@
       <c r="BK31" s="42"/>
       <c r="BL31" s="42"/>
     </row>
-    <row r="32" spans="1:64" s="30" customFormat="1" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="19"/>
       <c r="B32" s="50" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C32" s="51"/>
       <c r="D32" s="108"/>
@@ -4247,27 +4358,27 @@
       <c r="BK32" s="42"/>
       <c r="BL32" s="42"/>
     </row>
-    <row r="33" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="19"/>
       <c r="B33" s="57" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C33" s="58" t="s">
         <v>22</v>
       </c>
       <c r="D33" s="110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="59">
         <v>46216</v>
       </c>
       <c r="F33" s="111">
-        <v>46218</v>
+        <v>46222</v>
       </c>
       <c r="G33" s="28"/>
       <c r="H33" s="52">
-        <f t="shared" si="6"/>
-        <v>3</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>7</v>
       </c>
       <c r="I33" s="42"/>
       <c r="J33" s="42"/>
@@ -4326,27 +4437,27 @@
       <c r="BK33" s="42"/>
       <c r="BL33" s="42"/>
     </row>
-    <row r="34" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="19"/>
       <c r="B34" s="57" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="C34" s="58" t="s">
         <v>35</v>
       </c>
       <c r="D34" s="110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" s="59">
         <v>46217</v>
       </c>
       <c r="F34" s="111">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="G34" s="28"/>
       <c r="H34" s="52">
-        <f t="shared" si="6"/>
-        <v>3</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>6</v>
       </c>
       <c r="I34" s="42"/>
       <c r="J34" s="42"/>
@@ -4405,27 +4516,27 @@
       <c r="BK34" s="42"/>
       <c r="BL34" s="42"/>
     </row>
-    <row r="35" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:64" s="30" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="19"/>
       <c r="B35" s="57" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C35" s="58" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D35" s="110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" s="59">
         <v>46218</v>
       </c>
       <c r="F35" s="111">
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="G35" s="28"/>
       <c r="H35" s="52">
-        <f t="shared" si="6"/>
-        <v>3</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>5</v>
       </c>
       <c r="I35" s="42"/>
       <c r="J35" s="42"/>
@@ -4484,27 +4595,27 @@
       <c r="BK35" s="42"/>
       <c r="BL35" s="42"/>
     </row>
-    <row r="36" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="19"/>
       <c r="B36" s="57" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C36" s="58" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="D36" s="110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="59">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="F36" s="111">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="G36" s="28"/>
       <c r="H36" s="52">
-        <f t="shared" si="6"/>
-        <v>2</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>4</v>
       </c>
       <c r="I36" s="42"/>
       <c r="J36" s="42"/>
@@ -4563,26 +4674,27 @@
       <c r="BK36" s="42"/>
       <c r="BL36" s="42"/>
     </row>
-    <row r="37" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:64" s="30" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="19"/>
       <c r="B37" s="57" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="C37" s="58" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D37" s="110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" s="59">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="F37" s="111">
         <v>46222</v>
       </c>
       <c r="G37" s="28"/>
       <c r="H37" s="52">
-        <v>2</v>
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>3</v>
       </c>
       <c r="I37" s="42"/>
       <c r="J37" s="42"/>
@@ -4641,10 +4753,10 @@
       <c r="BK37" s="42"/>
       <c r="BL37" s="42"/>
     </row>
-    <row r="38" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="19"/>
       <c r="B38" s="90" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C38" s="94"/>
       <c r="D38" s="109"/>
@@ -4709,25 +4821,26 @@
       <c r="BK38" s="42"/>
       <c r="BL38" s="42"/>
     </row>
-    <row r="39" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:64" s="30" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="19"/>
       <c r="B39" s="97" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="C39" s="91" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D39" s="110">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="E39" s="92">
+        <v>46222</v>
+      </c>
+      <c r="F39" s="120">
         <v>46223</v>
-      </c>
-      <c r="F39" s="120">
-        <v>46224</v>
       </c>
       <c r="G39" s="28"/>
       <c r="H39" s="93">
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>2</v>
       </c>
       <c r="I39" s="42"/>
@@ -4787,16 +4900,16 @@
       <c r="BK39" s="42"/>
       <c r="BL39" s="42"/>
     </row>
-    <row r="40" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:64" s="30" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="19"/>
       <c r="B40" s="99" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="C40" s="91" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D40" s="110">
-        <v>0</v>
+        <v>0.65</v>
       </c>
       <c r="E40" s="92">
         <v>46223</v>
@@ -4806,6 +4919,7 @@
       </c>
       <c r="G40" s="28"/>
       <c r="H40" s="93">
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>3</v>
       </c>
       <c r="I40" s="42"/>
@@ -4865,16 +4979,16 @@
       <c r="BK40" s="42"/>
       <c r="BL40" s="42"/>
     </row>
-    <row r="41" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="19"/>
       <c r="B41" s="97" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C41" s="91" t="s">
         <v>22</v>
       </c>
       <c r="D41" s="110">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="E41" s="92">
         <v>46224</v>
@@ -4884,6 +4998,7 @@
       </c>
       <c r="G41" s="28"/>
       <c r="H41" s="93">
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>3</v>
       </c>
       <c r="I41" s="42"/>
@@ -4943,16 +5058,16 @@
       <c r="BK41" s="42"/>
       <c r="BL41" s="42"/>
     </row>
-    <row r="42" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="19"/>
       <c r="B42" s="97" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C42" s="91" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="110">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E42" s="92">
         <v>46225</v>
@@ -4962,6 +5077,7 @@
       </c>
       <c r="G42" s="28"/>
       <c r="H42" s="93">
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>3</v>
       </c>
       <c r="I42" s="42"/>
@@ -5021,16 +5137,16 @@
       <c r="BK42" s="42"/>
       <c r="BL42" s="42"/>
     </row>
-    <row r="43" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="19"/>
       <c r="B43" s="97" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="C43" s="91" t="s">
         <v>20</v>
       </c>
       <c r="D43" s="110">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E43" s="92">
         <v>46227</v>
@@ -5040,6 +5156,7 @@
       </c>
       <c r="G43" s="28"/>
       <c r="H43" s="93">
+        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>1</v>
       </c>
       <c r="I43" s="42"/>
@@ -5099,7 +5216,7 @@
       <c r="BK43" s="42"/>
       <c r="BL43" s="42"/>
     </row>
-    <row r="44" spans="1:64" s="30" customFormat="1" ht="11.25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:64" s="30" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="19"/>
       <c r="B44" s="40"/>
       <c r="C44" s="39"/>
@@ -5557,31 +5674,31 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B1"/>
     </row>
     <row r="2" spans="1:3" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="B4" s="104">
         <v>46188</v>
@@ -5589,63 +5706,63 @@
     </row>
     <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="7" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="7" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>13</v>

</xml_diff>